<commit_message>
fix: corrige TIPO, nombres de sedes en acumulado
</commit_message>
<xml_diff>
--- a/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO ATABANZA 503_Ajustado_20260625_102359.xlsx
+++ b/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO ATABANZA 503_Ajustado_20260625_102359.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\Ajustar 3 y 5\Ajustados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\PRUEBAS A CALIFICAR\Ya procesadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D14E835-108E-40AB-8C57-DF7DC0EA0105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="720" windowWidth="19190" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10" yWindow="380" windowWidth="19190" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultados" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
corrige Cod.Est en 3 archivos (SANTIAGO 301, MARGARITAS 501, ATABANZA 503)
</commit_message>
<xml_diff>
--- a/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO ATABANZA 503_Ajustado_20260625_102359.xlsx
+++ b/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO ATABANZA 503_Ajustado_20260625_102359.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\PRUEBAS A CALIFICAR\Ya procesadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D14E835-108E-40AB-8C57-DF7DC0EA0105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E19C45-C54C-47C0-BE38-2EE573B11369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="380" windowWidth="19190" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultados" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resultados!$A$1:$AB$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resultados!$A$1:$AB$35</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="72">
   <si>
     <t>Est.</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>1023021502</t>
+  </si>
+  <si>
+    <t>1140929606</t>
   </si>
 </sst>
 </file>
@@ -709,8 +712,8 @@
       <c r="D2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>31</v>
+      <c r="E2" t="s">
+        <v>71</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>32</v>
@@ -793,8 +796,8 @@
       <c r="D3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>31</v>
+      <c r="E3" t="s">
+        <v>71</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>32</v>
@@ -3609,7 +3612,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AB35" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>